<commit_message>
[FIX] ui size issue
</commit_message>
<xml_diff>
--- a/tests/fixtures/xlsx_test.xlsx
+++ b/tests/fixtures/xlsx_test.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E6"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -590,6 +590,546 @@
         </is>
       </c>
     </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>Tim</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>Berners-Lee</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>tim.bernerslee@example.com</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>14/03/2026</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>F1A4D7G2J5L8</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Barbara</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Liskov</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>barbara.liskov@example.com</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>G2B5E8H3K6M9</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Donald</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Knuth</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>donald.knuth@example.com</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>15/03/2026</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>H3C6F9J4L7N1</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Edsger</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Dijkstra</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>edsger.dijkstra@example.com</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>J4D7G1K5M8P2</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Linus</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>Torvalds</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>linus.torvalds@example.com</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>16/03/2026</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>K5E8H2L6N9Q3</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Ken</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Thompson</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ken.thompson@example.com</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>L6F9J3M7P1R4</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Dennis</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Ritchie</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>dennis.ritchie@example.com</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>17/03/2026</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>M7G1K4N8Q2S5</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Leslie</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Lamport</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>leslie.lamport@example.com</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>N8H2L5P9R3T6</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Niklaus</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Wirth</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>niklaus.wirth@example.com</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>18/03/2026</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>P9J3M6Q1S4U7</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Brian</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Kernighan</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>brian.kernighan@example.com</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Q1K4N7R2T5V8</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Bjarne</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Stroustrup</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>bjarne.stroustrup@example.com</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>19/03/2026</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>R2L5P8S3U6W9</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>James</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Gosling</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>james.gosling@example.com</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>S3M6Q9T4V7X1</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>Guido</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>van Rossum</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>guido.vanrossum@example.com</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>20/03/2026</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>T4N7R1U5W8Y2</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>Brendan</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Eich</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>brendan.eich@example.com</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>U5P8S2V6X9Z3</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>Anders</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Hejlsberg</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>anders.hejlsberg@example.com</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>21/03/2026</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>V6Q9T3W7Y1A4</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>Margaret</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Mitchell</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>margaret.mitchell@example.com</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>W7R1U4X8Z2B5</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>Yann</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>LeCun</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>yann.lecun@example.com</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>22/03/2026</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>X8S2V5Y9A3C6</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>Geoffrey</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Hinton</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>geoffrey.hinton@example.com</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Y9T3W6Z1B4D7</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Andrew</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Ng</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>andrew.ng@example.com</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>23/03/2026</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Z1U4X7A2C5E8</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>Fei-Fei</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Li</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>feifei.li@example.com</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>24/03/2026</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>A2V5Y8B3D6F9</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>